<commit_message>
docs: richer Northwind FY2026 demo screenshots
Replace sparse README previews with a multi-sheet English operating-plan workbook and regenerated assets (including Pipeline).
</commit_message>
<xml_diff>
--- a/examples/demo_budget.xlsx
+++ b/examples/demo_budget.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="By region" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Charts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="By segment" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pipeline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,11 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$#,##0;($#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,7 +37,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001E2761"/>
+      <color rgb="001E3A5F"/>
       <sz val="16"/>
     </font>
     <font>
@@ -67,13 +70,25 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001F2430"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="006B7280"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001E2761"/>
+      <color rgb="001E3A5F"/>
       <sz val="18"/>
     </font>
     <font>
@@ -102,7 +117,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E2761"/>
+        <fgColor rgb="001E3A5F"/>
       </patternFill>
     </fill>
     <fill>
@@ -161,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -170,6 +185,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,19 +214,55 @@
     <xf numFmtId="165" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="10" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C8E6C9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -309,7 +363,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Charts'!B7</f>
+              <f>'Dashboard'!AO7</f>
             </strRef>
           </tx>
           <spPr>
@@ -319,12 +373,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Charts'!$A$8:$A$10</f>
+              <f>'Dashboard'!$AN$8:$AN$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$B$8:$B$10</f>
+              <f>'Dashboard'!$AO$8:$AO$11</f>
             </numRef>
           </val>
         </ser>
@@ -350,6 +404,21 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>USD</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -377,7 +446,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue mix by region (Q3)</a:t>
+              <a:t>FY mix by segment</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -391,7 +460,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Charts'!B12</f>
+              <f>'Dashboard'!AO23</f>
             </strRef>
           </tx>
           <spPr>
@@ -401,12 +470,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Charts'!$A$13:$A$15</f>
+              <f>'Dashboard'!$AN$24:$AN$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$B$13:$B$15</f>
+              <f>'Dashboard'!$AO$24:$AO$27</f>
             </numRef>
           </val>
         </ser>
@@ -416,7 +485,7 @@
           <showPercent val="1"/>
         </dLbls>
         <firstSliceAng val="0"/>
-        <holeSize val="10"/>
+        <holeSize val="50"/>
       </doughnutChart>
     </plotArea>
     <legend>
@@ -436,7 +505,7 @@
   <commentList>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Source: board pack Q2</t>
+        <t>Source: board pack Q4 FY2025</t>
       </text>
     </comment>
   </commentList>
@@ -452,7 +521,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2880000"/>
+    <ext cx="5040000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -469,12 +538,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2880000"/>
+    <ext cx="4320000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -493,27 +562,46 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PnL" displayName="PnL" ref="A3:E8" headerRowCount="1">
-  <autoFilter ref="A3:E8"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PnL" displayName="PnL" ref="A3:F12" headerRowCount="1">
+  <autoFilter ref="A3:F12"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="Line item"/>
     <tableColumn id="2" name="Q1"/>
     <tableColumn id="3" name="Q2"/>
     <tableColumn id="4" name="Q3"/>
-    <tableColumn id="5" name="Total"/>
+    <tableColumn id="5" name="Q4"/>
+    <tableColumn id="6" name="FY Total"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="By_region" displayName="By_region" ref="A3:D6" headerRowCount="1">
-  <autoFilter ref="A3:D6"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Region"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="By_segment" displayName="By_segment" ref="A3:F7" headerRowCount="1">
+  <autoFilter ref="A3:F7"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Segment"/>
     <tableColumn id="2" name="Q1"/>
     <tableColumn id="3" name="Q2"/>
     <tableColumn id="4" name="Q3"/>
+    <tableColumn id="5" name="Q4"/>
+    <tableColumn id="6" name="FY"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Pipeline" displayName="Pipeline" ref="A3:G10" headerRowCount="1">
+  <autoFilter ref="A3:G10"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Opportunity"/>
+    <tableColumn id="2" name="Owner"/>
+    <tableColumn id="3" name="Stage"/>
+    <tableColumn id="4" name="Amount"/>
+    <tableColumn id="5" name="Win %"/>
+    <tableColumn id="6" name="Weighted"/>
+    <tableColumn id="7" name="Close"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -805,11 +893,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001E2761"/>
+    <tabColor rgb="001E3A5F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -821,14 +909,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Key assumptions</t>
+          <t>Planning assumptions</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Yellow cells with blue text are inputs — edit these. Other sheets reference them with formulas.</t>
+          <t>Yellow cells with blue text are editable inputs. Downstream sheets reference these values with formulas.</t>
         </is>
       </c>
     </row>
@@ -857,11 +945,11 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Revenue growth</t>
+          <t>Revenue growth YoY</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -870,7 +958,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>YoY</t>
+          <t>Base case</t>
         </is>
       </c>
     </row>
@@ -893,7 +981,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Tax rate</t>
+          <t>Effective tax rate</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -909,18 +997,66 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Headcount</t>
+          <t>Avg billable day rate</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>42</v>
+        <v>850</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Billable days / FTE / year</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Headcount (end of year)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
           <t>FTE</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Fixed OpEx / month</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>42000</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -935,151 +1071,291 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001E2761"/>
+    <tabColor rgb="001E3A5F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Profit &amp; Loss — quarterly</t>
+          <t>Consolidated P&amp;L — quarterly</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Line item</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>FY Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Software &amp; platform revenue</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>420000</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>455000</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>510000</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>580000</v>
+      </c>
+      <c r="F4" s="11">
+        <f>SUM(B4:E4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Professional services</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>185000</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>198000</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>215000</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>240000</v>
+      </c>
+      <c r="F5" s="14">
+        <f>SUM(B5:E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Marketplace &amp; licenses</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>62000</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>71000</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>78000</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>92000</v>
+      </c>
+      <c r="F6" s="11">
+        <f>SUM(B6:E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Cost of delivery</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>-210000</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>-225000</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>-248000</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>-275000</v>
+      </c>
+      <c r="F7" s="14">
+        <f>SUM(B7:E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Cloud infrastructure</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>-48000</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>-51000</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>-55000</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>-61000</v>
+      </c>
+      <c r="F8" s="11">
+        <f>SUM(B8:E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Sales &amp; marketing</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>-95000</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>-102000</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>-118000</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>-130000</v>
+      </c>
+      <c r="F9" s="14">
+        <f>SUM(B9:E9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>R&amp;D / product</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>-140000</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>-145000</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>-152000</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>-160000</v>
+      </c>
+      <c r="F10" s="11">
+        <f>SUM(B10:E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>G&amp;A</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>-72000</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>-74000</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>-76000</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>-78000</v>
+      </c>
+      <c r="F11" s="14">
+        <f>SUM(B11:E11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; amortisation</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>-19000</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>-19000</v>
+      </c>
+      <c r="F12" s="11">
+        <f>SUM(B12:E12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="n">
-        <v>120000</v>
-      </c>
-      <c r="C4" s="9" t="n">
-        <v>135000</v>
-      </c>
-      <c r="D4" s="9" t="n">
-        <v>148000</v>
-      </c>
-      <c r="E4" s="10">
-        <f>SUM(B4:D4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>COGS</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>48000</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>52000</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>56000</v>
-      </c>
-      <c r="E5" s="13">
-        <f>SUM(B5:D5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Gross profit</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="n">
-        <v>72000</v>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>83000</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>92000</v>
-      </c>
-      <c r="E6" s="10">
-        <f>SUM(B6:D6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>OpEx</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>30000</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>31000</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>33000</v>
-      </c>
-      <c r="E7" s="13">
-        <f>SUM(B7:D7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Operating income</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>42000</v>
-      </c>
-      <c r="C8" s="9" t="n">
-        <v>52000</v>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>59000</v>
-      </c>
-      <c r="E8" s="10">
-        <f>SUM(B8:D8)</f>
+      <c r="B13" s="16">
+        <f>SUM(B4:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="16">
+        <f>SUM(C4:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="16">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="16">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="16">
+        <f>SUM(F4:F12)</f>
         <v/>
       </c>
     </row>
@@ -1087,38 +1363,51 @@
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B4:B8">
+  <conditionalFormatting sqref="B4:B12">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="002E5AAC"/>
+        <color rgb="001E3A5F"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C8">
+  <conditionalFormatting sqref="C4:C12">
     <cfRule type="dataBar" priority="2">
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="002E5AAC"/>
+        <color rgb="001E3A5F"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D8">
+  <conditionalFormatting sqref="D4:D12">
     <cfRule type="dataBar" priority="3">
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="002E5AAC"/>
+        <color rgb="001E3A5F"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="A4:A8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Validation" error="Invalid value" type="list">
-      <formula1>"Revenue,COGS,Gross profit,OpEx,Operating income,Other"</formula1>
-    </dataValidation>
-  </dataValidations>
+  <conditionalFormatting sqref="E4:E12">
+    <cfRule type="dataBar" priority="4">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="001E3A5F"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F4:F12">
+    <cfRule type="dataBar" priority="5">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="002E7D32"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1129,100 +1418,216 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001E2761"/>
+    <tabColor rgb="001E3A5F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Revenue by region</t>
+          <t>Revenue by segment × quarter</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>FY</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>EMEA</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="n">
-        <v>52000</v>
-      </c>
-      <c r="C4" s="9" t="n">
-        <v>58000</v>
-      </c>
-      <c r="D4" s="9" t="n">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>310000</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>335000</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>380000</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>425000</v>
+      </c>
+      <c r="F4" s="11">
+        <f>SUM(B4:E4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Mid-market</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>215000</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>238000</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>265000</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>298000</v>
+      </c>
+      <c r="F5" s="14">
+        <f>SUM(B5:E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>SMB / self-serve</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>92000</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>101000</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>112000</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>128000</v>
+      </c>
+      <c r="F6" s="11">
+        <f>SUM(B6:E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Partner channel</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>46000</v>
+      </c>
+      <c r="E7" s="13" t="n">
         <v>61000</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Americas</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>40000</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>51000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>APAC</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="n">
-        <v>28000</v>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>32000</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>36000</v>
+      <c r="F7" s="14">
+        <f>SUM(B7:E7)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B4:B7">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:C7">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D7">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4:E7">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F4:F7">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1233,169 +1638,529 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001E2761"/>
+    <tabColor rgb="001E3A5F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sales pipeline — weighted</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Opportunity</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Win %</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Weighted</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Acme Corp — platform rollout</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>M. Chen</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Negotiate</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>280000</v>
+      </c>
+      <c r="E4" s="17" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F4" s="11">
+        <f>D4*E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="18" t="n">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Globex AI copilot suite</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>J. Patel</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>145000</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F5" s="14">
+        <f>D5*E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>46172</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Initech multi-year MSA</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>M. Chen</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Qualify</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>420000</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F6" s="11">
+        <f>D6*E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Umbrella regional expansion</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>S. Okonkwo</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Negotiate</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>96000</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F7" s="14">
+        <f>D7*E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Stark Industries SOC2 pack</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>J. Patel</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Closed Won</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>72000</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="11">
+        <f>D8*E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="18" t="n">
+        <v>46063</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Wayne Health LLM pilot</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>S. Okonkwo</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>118000</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F9" s="14">
+        <f>D9*E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Oscorp data platform</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>M. Chen</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Qualify</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>195000</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F10" s="11">
+        <f>D10*E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="18" t="n">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="16">
+        <f>SUM(D4:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="16">
+        <f>SUM(F4:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="23" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F4:F10">
+    <cfRule type="dataBar" priority="1">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="002E7D32"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4:E10">
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Validation" error="Invalid value" type="list">
+      <formula1>"Qualify,Proposal,Negotiate,Closed Won,Closed Lost"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001E3A5F"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AO40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Highlights</t>
+          <t>FY2026 highlights</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>YTD REVENUE</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>FY REVENUE</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>GROSS MARGIN</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>OP. INCOME</t>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>PIPELINE WEIGHTED</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>HEADCOUNT</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="n">
-        <v>403000</v>
-      </c>
-      <c r="B4" s="16" t="n">
+      <c r="A4" s="25" t="n">
+        <v>2417000</v>
+      </c>
+      <c r="B4" s="26" t="n">
         <v>0.61</v>
       </c>
-      <c r="C4" s="15" t="n">
-        <v>153000</v>
+      <c r="C4" s="25" t="n">
+        <v>612100</v>
+      </c>
+      <c r="D4" s="27" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>+12% YoY</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>+2 pp</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n"/>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>7 deals</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>+6 FTE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="AN7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Value</t>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>Revenue</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="AN8" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>120000</v>
+      <c r="AO8" t="n">
+        <v>667000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="AN9" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>135000</v>
+      <c r="AO9" t="n">
+        <v>724000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="AN10" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>148000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="AO10" t="n">
+        <v>803000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="AO11" t="n">
+        <v>912000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="AN23" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>EMEA</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>61000</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Americas</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>51000</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>APAC</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>36000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>FY mix</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="AO24" t="n">
+        <v>1450000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Mid-market</t>
+        </is>
+      </c>
+      <c r="AO25" t="n">
+        <v>1016000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>SMB</t>
+        </is>
+      </c>
+      <c r="AO26" t="n">
+        <v>433000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="AO27" t="n">
+        <v>207000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
         <is>
           <t>How to use this workbook</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Edit yellow input cells on the Assumptions sheet. P&amp;L totals are live Excel formulas (=SUM). Open in Excel or LibreOffice to recalculate.</t>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>1) Edit yellow inputs on Assumptions. 2) P&amp;L and Pipeline FY/Weighted columns are live Excel formulas. 3) Open in Excel or LibreOffice to recalculate cached values. Figures are illustrative for the Generate Spreadsheets demo.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A39:D39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>